<commit_message>
Except BSL all Techno db backend code written DSP under testing
</commit_message>
<xml_diff>
--- a/Report_format/Monthly/BSPOISCO_MAY'25.xlsx
+++ b/Report_format/Monthly/BSPOISCO_MAY'25.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\opr-mis1\Report_format\Monthly\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ADC76A0C-8749-4CE9-A978-F794412F1689}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="315" windowWidth="11115" windowHeight="5640"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -205,10 +211,10 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="186" formatCode="0.000"/>
-    <numFmt numFmtId="187" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -577,7 +583,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -585,7 +591,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -599,7 +605,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -618,10 +624,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="187" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="187" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -633,25 +639,19 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="187" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="187" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="187" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="187" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="187" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="187" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -666,12 +666,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="187" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="187" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -684,16 +678,16 @@
     <xf numFmtId="1" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="187" fontId="5" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="187" fontId="4" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -714,13 +708,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="187" fontId="5" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="5" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -741,10 +732,10 @@
     <xf numFmtId="2" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="186" fontId="4" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="186" fontId="5" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -775,10 +766,10 @@
     <xf numFmtId="2" fontId="4" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="187" fontId="5" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="187" fontId="4" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -802,7 +793,7 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="186" fontId="5" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -811,14 +802,17 @@
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal_BOFTEC" xfId="1"/>
-    <cellStyle name="Normal_IRON" xfId="2"/>
+    <cellStyle name="Normal_BOFTEC" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Normal_IRON" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1195,42 +1189,42 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:H58"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="1.6640625" customWidth="1"/>
+    <col min="2" max="2" width="9.109375" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="4" max="4" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.85546875" customWidth="1"/>
-    <col min="7" max="7" width="8.28515625" customWidth="1"/>
+    <col min="4" max="4" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.88671875" customWidth="1"/>
+    <col min="7" max="7" width="8.33203125" customWidth="1"/>
     <col min="8" max="8" width="33" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="2" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
-      <c r="H2" s="71" t="s">
+      <c r="H2" s="66" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="3:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="C3" s="79" t="s">
+    <row r="3" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C3" s="74" t="s">
         <v>58</v>
       </c>
-      <c r="D3" s="79"/>
-      <c r="E3" s="79"/>
-      <c r="F3" s="79"/>
-      <c r="G3" s="79"/>
-      <c r="H3" s="79"/>
-    </row>
-    <row r="4" spans="3:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="D3" s="74"/>
+      <c r="E3" s="74"/>
+      <c r="F3" s="74"/>
+      <c r="G3" s="74"/>
+      <c r="H3" s="74"/>
+    </row>
+    <row r="4" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="C4" s="3"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
@@ -1238,7 +1232,7 @@
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
     </row>
-    <row r="5" spans="3:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="3:8" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C5" s="4" t="s">
         <v>31</v>
       </c>
@@ -1246,7 +1240,7 @@
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
     </row>
-    <row r="6" spans="3:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:8" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="s">
         <v>24</v>
@@ -1264,7 +1258,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="3:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="7" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="C7" s="11"/>
       <c r="D7" s="12"/>
       <c r="E7" s="13"/>
@@ -1272,21 +1266,21 @@
       <c r="G7" s="13"/>
       <c r="H7" s="14"/>
     </row>
-    <row r="8" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C8" s="42" t="s">
+    <row r="8" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C8" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="D8" s="46"/>
-      <c r="E8" s="43"/>
-      <c r="F8" s="43"/>
-      <c r="G8" s="43"/>
-      <c r="H8" s="44"/>
-    </row>
-    <row r="9" spans="3:8" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="C9" s="28" t="s">
+      <c r="D8" s="42"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="40"/>
+    </row>
+    <row r="9" spans="3:8" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="C9" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="45" t="s">
+      <c r="D9" s="41" t="s">
         <v>46</v>
       </c>
       <c r="E9" s="21">
@@ -1300,65 +1294,65 @@
       </c>
       <c r="H9" s="23"/>
     </row>
-    <row r="10" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C10" s="29" t="s">
+    <row r="10" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C10" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="D10" s="45" t="s">
+      <c r="D10" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="E10" s="26" t="s">
+      <c r="E10" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="F10" s="26" t="s">
+      <c r="F10" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="G10" s="27" t="s">
+      <c r="G10" s="25" t="s">
         <v>7</v>
       </c>
       <c r="H10" s="23"/>
     </row>
-    <row r="11" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C11" s="29" t="s">
+    <row r="11" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C11" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="45" t="s">
+      <c r="D11" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="26">
+      <c r="E11" s="24">
         <v>105.18945408749931</v>
       </c>
-      <c r="F11" s="26">
+      <c r="F11" s="24">
         <v>113.65230928905034</v>
       </c>
-      <c r="G11" s="27">
+      <c r="G11" s="25">
         <v>109.53440971944687</v>
       </c>
-      <c r="H11" s="30"/>
-    </row>
-    <row r="12" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C12" s="29" t="s">
+      <c r="H11" s="28"/>
+    </row>
+    <row r="12" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C12" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="D12" s="45" t="s">
+      <c r="D12" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="E12" s="26" t="s">
+      <c r="E12" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="F12" s="26" t="s">
+      <c r="F12" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="G12" s="27" t="s">
+      <c r="G12" s="25" t="s">
         <v>7</v>
       </c>
       <c r="H12" s="23"/>
     </row>
-    <row r="13" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C13" s="29" t="s">
+    <row r="13" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C13" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="D13" s="45" t="s">
+      <c r="D13" s="41" t="s">
         <v>46</v>
       </c>
       <c r="E13" s="24">
@@ -1370,49 +1364,49 @@
       <c r="G13" s="25">
         <v>106.1988208525563</v>
       </c>
-      <c r="H13" s="31"/>
-    </row>
-    <row r="14" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C14" s="29" t="s">
+      <c r="H13" s="29"/>
+    </row>
+    <row r="14" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C14" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="D14" s="45" t="s">
+      <c r="D14" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="E14" s="26">
+      <c r="E14" s="24">
         <v>82.039971701450298</v>
       </c>
-      <c r="F14" s="26">
+      <c r="F14" s="24">
         <v>103.16571401008127</v>
       </c>
-      <c r="G14" s="27">
+      <c r="G14" s="25">
         <v>96.563956026949811</v>
       </c>
-      <c r="H14" s="31"/>
-    </row>
-    <row r="15" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C15" s="29" t="s">
+      <c r="H14" s="29"/>
+    </row>
+    <row r="15" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C15" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="D15" s="45" t="s">
+      <c r="D15" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="E15" s="26">
+      <c r="E15" s="24">
         <v>137.51414873982401</v>
       </c>
-      <c r="F15" s="26">
+      <c r="F15" s="24">
         <v>134.53519188823654</v>
       </c>
-      <c r="G15" s="27">
+      <c r="G15" s="25">
         <v>136.04002089055669</v>
       </c>
-      <c r="H15" s="31"/>
-    </row>
-    <row r="16" spans="3:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="H15" s="29"/>
+    </row>
+    <row r="16" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="C16" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="D16" s="45" t="s">
+      <c r="D16" s="41" t="s">
         <v>46</v>
       </c>
       <c r="E16" s="21">
@@ -1424,13 +1418,13 @@
       <c r="G16" s="22">
         <v>561.4258111343122</v>
       </c>
-      <c r="H16" s="31"/>
-    </row>
-    <row r="17" spans="3:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="H16" s="29"/>
+    </row>
+    <row r="17" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="C17" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="D17" s="45" t="s">
+      <c r="D17" s="41" t="s">
         <v>5</v>
       </c>
       <c r="E17" s="21">
@@ -1442,13 +1436,13 @@
       <c r="G17" s="22">
         <v>14.545817667033859</v>
       </c>
-      <c r="H17" s="31"/>
-    </row>
-    <row r="18" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C18" s="29" t="s">
+      <c r="H17" s="29"/>
+    </row>
+    <row r="18" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C18" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="D18" s="45" t="s">
+      <c r="D18" s="41" t="s">
         <v>46</v>
       </c>
       <c r="E18" s="21">
@@ -1460,59 +1454,59 @@
       <c r="G18" s="22">
         <v>0</v>
       </c>
-      <c r="H18" s="31"/>
-    </row>
-    <row r="19" spans="3:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="H18" s="29"/>
+    </row>
+    <row r="19" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="C19" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="D19" s="45" t="s">
+      <c r="D19" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="E19" s="32">
+      <c r="E19" s="21">
         <v>0.2</v>
       </c>
-      <c r="F19" s="32">
+      <c r="F19" s="21">
         <v>0.18083182640144665</v>
       </c>
-      <c r="G19" s="33">
+      <c r="G19" s="22">
         <v>0.19958621887757921</v>
       </c>
-      <c r="H19" s="31"/>
-    </row>
-    <row r="20" spans="3:8" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="C20" s="50" t="s">
+      <c r="H19" s="29"/>
+    </row>
+    <row r="20" spans="3:8" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="C20" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="D20" s="45" t="s">
+      <c r="D20" s="41" t="s">
         <v>7</v>
       </c>
-      <c r="E20" s="58">
+      <c r="E20" s="53">
         <v>0.92200000000000004</v>
       </c>
-      <c r="F20" s="78"/>
-      <c r="G20" s="57">
+      <c r="F20" s="73"/>
+      <c r="G20" s="52">
         <v>0.92200000000000004</v>
       </c>
-      <c r="H20" s="51" t="s">
+      <c r="H20" s="46" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C21" s="42" t="s">
+    <row r="21" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C21" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="D21" s="46"/>
-      <c r="E21" s="43"/>
-      <c r="F21" s="43"/>
-      <c r="G21" s="43"/>
-      <c r="H21" s="44"/>
-    </row>
-    <row r="22" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C22" s="34" t="s">
+      <c r="D21" s="42"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="39"/>
+      <c r="G21" s="39"/>
+      <c r="H21" s="40"/>
+    </row>
+    <row r="22" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C22" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="D22" s="45" t="s">
+      <c r="D22" s="41" t="s">
         <v>10</v>
       </c>
       <c r="E22" s="21">
@@ -1524,13 +1518,13 @@
       <c r="G22" s="22">
         <v>82.4</v>
       </c>
-      <c r="H22" s="31"/>
-    </row>
-    <row r="23" spans="3:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="H22" s="29"/>
+    </row>
+    <row r="23" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="C23" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D23" s="45" t="s">
+      <c r="D23" s="41" t="s">
         <v>50</v>
       </c>
       <c r="E23" s="21">
@@ -1542,13 +1536,13 @@
       <c r="G23" s="22">
         <v>76.3</v>
       </c>
-      <c r="H23" s="31"/>
-    </row>
-    <row r="24" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C24" s="34" t="s">
+      <c r="H23" s="29"/>
+    </row>
+    <row r="24" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C24" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="D24" s="45" t="s">
+      <c r="D24" s="41" t="s">
         <v>13</v>
       </c>
       <c r="E24" s="21">
@@ -1560,13 +1554,13 @@
       <c r="G24" s="22">
         <v>54.57</v>
       </c>
-      <c r="H24" s="31"/>
-    </row>
-    <row r="25" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C25" s="34" t="s">
+      <c r="H24" s="29"/>
+    </row>
+    <row r="25" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C25" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="D25" s="45" t="s">
+      <c r="D25" s="41" t="s">
         <v>48</v>
       </c>
       <c r="E25" s="21">
@@ -1578,13 +1572,13 @@
       <c r="G25" s="22">
         <v>49.803278688524593</v>
       </c>
-      <c r="H25" s="31"/>
-    </row>
-    <row r="26" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C26" s="34" t="s">
+      <c r="H25" s="29"/>
+    </row>
+    <row r="26" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C26" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="D26" s="45" t="s">
+      <c r="D26" s="41" t="s">
         <v>49</v>
       </c>
       <c r="E26" s="21">
@@ -1596,49 +1590,49 @@
       <c r="G26" s="22">
         <v>120.18861092824227</v>
       </c>
-      <c r="H26" s="31"/>
-    </row>
-    <row r="27" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C27" s="34" t="s">
+      <c r="H26" s="29"/>
+    </row>
+    <row r="27" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C27" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="D27" s="45" t="s">
+      <c r="D27" s="41" t="s">
         <v>48</v>
       </c>
-      <c r="E27" s="35">
+      <c r="E27" s="31">
         <v>6494</v>
       </c>
-      <c r="F27" s="36" t="s">
+      <c r="F27" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="G27" s="37">
+      <c r="G27" s="33">
         <v>6494</v>
       </c>
-      <c r="H27" s="31"/>
-    </row>
-    <row r="28" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C28" s="34" t="s">
+      <c r="H27" s="29"/>
+    </row>
+    <row r="28" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C28" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="D28" s="45" t="s">
+      <c r="D28" s="41" t="s">
         <v>45</v>
       </c>
-      <c r="E28" s="38">
+      <c r="E28" s="34">
         <v>0</v>
       </c>
-      <c r="F28" s="38">
+      <c r="F28" s="34">
         <v>0</v>
       </c>
-      <c r="G28" s="39">
+      <c r="G28" s="35">
         <v>0</v>
       </c>
-      <c r="H28" s="31"/>
-    </row>
-    <row r="29" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C29" s="34" t="s">
+      <c r="H28" s="29"/>
+    </row>
+    <row r="29" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C29" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="D29" s="45" t="s">
+      <c r="D29" s="41" t="s">
         <v>45</v>
       </c>
       <c r="E29" s="21">
@@ -1650,13 +1644,13 @@
       <c r="G29" s="22">
         <v>1.647</v>
       </c>
-      <c r="H29" s="31"/>
-    </row>
-    <row r="30" spans="3:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="H29" s="29"/>
+    </row>
+    <row r="30" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="C30" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="D30" s="45" t="s">
+      <c r="D30" s="41" t="s">
         <v>45</v>
       </c>
       <c r="E30" s="21">
@@ -1668,13 +1662,13 @@
       <c r="G30" s="22">
         <v>17.547000000000001</v>
       </c>
-      <c r="H30" s="31"/>
-    </row>
-    <row r="31" spans="3:8" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="C31" s="28" t="s">
+      <c r="H30" s="29"/>
+    </row>
+    <row r="31" spans="3:8" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="C31" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="D31" s="45" t="s">
+      <c r="D31" s="41" t="s">
         <v>47</v>
       </c>
       <c r="E31" s="21">
@@ -1686,31 +1680,31 @@
       <c r="G31" s="22">
         <v>70.62338654681993</v>
       </c>
-      <c r="H31" s="31"/>
-    </row>
-    <row r="32" spans="3:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="H31" s="29"/>
+    </row>
+    <row r="32" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="C32" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="D32" s="45" t="s">
+      <c r="D32" s="41" t="s">
         <v>45</v>
       </c>
-      <c r="E32" s="32">
+      <c r="E32" s="21">
         <v>0.35399999999999998</v>
       </c>
-      <c r="F32" s="32">
+      <c r="F32" s="21">
         <v>0.33899999999999997</v>
       </c>
-      <c r="G32" s="33">
+      <c r="G32" s="22">
         <v>0.35099999999999998</v>
       </c>
-      <c r="H32" s="31"/>
-    </row>
-    <row r="33" spans="3:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="H32" s="29"/>
+    </row>
+    <row r="33" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="C33" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="D33" s="47" t="s">
+      <c r="D33" s="43" t="s">
         <v>45</v>
       </c>
       <c r="E33" s="16">
@@ -1724,11 +1718,11 @@
       </c>
       <c r="H33" s="18"/>
     </row>
-    <row r="34" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C34" s="52" t="s">
+    <row r="34" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C34" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="D34" s="53" t="s">
+      <c r="D34" s="48" t="s">
         <v>45</v>
       </c>
       <c r="E34" s="21">
@@ -1740,13 +1734,13 @@
       <c r="G34" s="22">
         <v>0.246</v>
       </c>
-      <c r="H34" s="31"/>
-    </row>
-    <row r="35" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C35" s="52" t="s">
+      <c r="H34" s="29"/>
+    </row>
+    <row r="35" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C35" s="47" t="s">
         <v>54</v>
       </c>
-      <c r="D35" s="53" t="s">
+      <c r="D35" s="48" t="s">
         <v>55</v>
       </c>
       <c r="E35" s="21">
@@ -1758,41 +1752,41 @@
       <c r="G35" s="22">
         <v>26.6</v>
       </c>
-      <c r="H35" s="31"/>
-    </row>
-    <row r="36" spans="3:8" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="C36" s="60" t="s">
+      <c r="H35" s="29"/>
+    </row>
+    <row r="36" spans="3:8" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="C36" s="55" t="s">
         <v>56</v>
       </c>
-      <c r="D36" s="53" t="s">
+      <c r="D36" s="48" t="s">
         <v>57</v>
       </c>
-      <c r="E36" s="35">
+      <c r="E36" s="31">
         <v>0</v>
       </c>
-      <c r="F36" s="35">
+      <c r="F36" s="31">
         <v>0</v>
       </c>
-      <c r="G36" s="37">
+      <c r="G36" s="33">
         <v>0</v>
       </c>
-      <c r="H36" s="31"/>
-    </row>
-    <row r="37" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C37" s="42" t="s">
+      <c r="H36" s="29"/>
+    </row>
+    <row r="37" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C37" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="D37" s="46"/>
-      <c r="E37" s="43"/>
-      <c r="F37" s="43"/>
-      <c r="G37" s="43"/>
-      <c r="H37" s="44"/>
-    </row>
-    <row r="38" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C38" s="34" t="s">
+      <c r="D37" s="42"/>
+      <c r="E37" s="39"/>
+      <c r="F37" s="39"/>
+      <c r="G37" s="39"/>
+      <c r="H37" s="40"/>
+    </row>
+    <row r="38" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C38" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="D38" s="45" t="s">
+      <c r="D38" s="41" t="s">
         <v>10</v>
       </c>
       <c r="E38" s="21">
@@ -1804,13 +1798,13 @@
       <c r="G38" s="22">
         <v>80.094869459623553</v>
       </c>
-      <c r="H38" s="31"/>
-    </row>
-    <row r="39" spans="3:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="H38" s="29"/>
+    </row>
+    <row r="39" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="C39" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D39" s="45" t="s">
+      <c r="D39" s="41" t="s">
         <v>50</v>
       </c>
       <c r="E39" s="21">
@@ -1822,31 +1816,31 @@
       <c r="G39" s="22">
         <v>91.21517215376447</v>
       </c>
-      <c r="H39" s="31"/>
-    </row>
-    <row r="40" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C40" s="34" t="s">
+      <c r="H39" s="29"/>
+    </row>
+    <row r="40" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C40" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="D40" s="45" t="s">
+      <c r="D40" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="E40" s="40">
+      <c r="E40" s="36">
         <v>52.86</v>
       </c>
-      <c r="F40" s="40">
+      <c r="F40" s="36">
         <v>52.6</v>
       </c>
-      <c r="G40" s="41">
+      <c r="G40" s="37">
         <v>52.730000000000004</v>
       </c>
-      <c r="H40" s="31"/>
-    </row>
-    <row r="41" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C41" s="34" t="s">
+      <c r="H40" s="29"/>
+    </row>
+    <row r="41" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C41" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="D41" s="45" t="s">
+      <c r="D41" s="41" t="s">
         <v>48</v>
       </c>
       <c r="E41" s="21">
@@ -1858,13 +1852,13 @@
       <c r="G41" s="22">
         <v>59.868852459016395</v>
       </c>
-      <c r="H41" s="31"/>
-    </row>
-    <row r="42" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C42" s="34" t="s">
+      <c r="H41" s="29"/>
+    </row>
+    <row r="42" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C42" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="D42" s="45" t="s">
+      <c r="D42" s="41" t="s">
         <v>49</v>
       </c>
       <c r="E42" s="21">
@@ -1876,31 +1870,31 @@
       <c r="G42" s="22">
         <v>167.83710405257392</v>
       </c>
-      <c r="H42" s="31"/>
-    </row>
-    <row r="43" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C43" s="34" t="s">
+      <c r="H42" s="29"/>
+    </row>
+    <row r="43" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C43" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="D43" s="45" t="s">
+      <c r="D43" s="41" t="s">
         <v>45</v>
       </c>
-      <c r="E43" s="38">
+      <c r="E43" s="34">
         <v>0.16844259776305584</v>
       </c>
-      <c r="F43" s="38">
+      <c r="F43" s="34">
         <v>0.11482127494978234</v>
       </c>
-      <c r="G43" s="39">
+      <c r="G43" s="35">
         <v>0.13876212461044354</v>
       </c>
-      <c r="H43" s="31"/>
-    </row>
-    <row r="44" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C44" s="34" t="s">
+      <c r="H43" s="29"/>
+    </row>
+    <row r="44" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C44" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="D44" s="45" t="s">
+      <c r="D44" s="41" t="s">
         <v>45</v>
       </c>
       <c r="E44" s="21">
@@ -1912,13 +1906,13 @@
       <c r="G44" s="22">
         <v>2.4475698627277249</v>
       </c>
-      <c r="H44" s="31"/>
-    </row>
-    <row r="45" spans="3:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="H44" s="29"/>
+    </row>
+    <row r="45" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="C45" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="D45" s="45" t="s">
+      <c r="D45" s="41" t="s">
         <v>45</v>
       </c>
       <c r="E45" s="21">
@@ -1930,13 +1924,13 @@
       <c r="G45" s="22">
         <v>14.766516700147235</v>
       </c>
-      <c r="H45" s="31"/>
-    </row>
-    <row r="46" spans="3:8" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="C46" s="28" t="s">
+      <c r="H45" s="29"/>
+    </row>
+    <row r="46" spans="3:8" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="C46" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="D46" s="45" t="s">
+      <c r="D46" s="41" t="s">
         <v>47</v>
       </c>
       <c r="E46" s="21">
@@ -1948,31 +1942,31 @@
       <c r="G46" s="22">
         <v>62.450447922393835</v>
       </c>
-      <c r="H46" s="31"/>
-    </row>
-    <row r="47" spans="3:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="H46" s="29"/>
+    </row>
+    <row r="47" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="C47" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="D47" s="45" t="s">
+      <c r="D47" s="41" t="s">
         <v>45</v>
       </c>
-      <c r="E47" s="32">
+      <c r="E47" s="21">
         <v>0.37856374879607319</v>
       </c>
-      <c r="F47" s="32">
+      <c r="F47" s="21">
         <v>0.39336809104625603</v>
       </c>
-      <c r="G47" s="33">
+      <c r="G47" s="22">
         <v>0.38675824791778951</v>
       </c>
-      <c r="H47" s="31"/>
-    </row>
-    <row r="48" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C48" s="34" t="s">
+      <c r="H47" s="29"/>
+    </row>
+    <row r="48" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C48" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="D48" s="45" t="s">
+      <c r="D48" s="41" t="s">
         <v>45</v>
       </c>
       <c r="E48" s="21">
@@ -1984,13 +1978,13 @@
       <c r="G48" s="22">
         <v>71.25878779272395</v>
       </c>
-      <c r="H48" s="31"/>
-    </row>
-    <row r="49" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C49" s="52" t="s">
+      <c r="H48" s="29"/>
+    </row>
+    <row r="49" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C49" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="D49" s="53" t="s">
+      <c r="D49" s="48" t="s">
         <v>45</v>
       </c>
       <c r="E49" s="21">
@@ -2002,125 +1996,125 @@
       <c r="G49" s="22">
         <v>0</v>
       </c>
-      <c r="H49" s="31"/>
-    </row>
-    <row r="50" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C50" s="52" t="s">
+      <c r="H49" s="29"/>
+    </row>
+    <row r="50" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C50" s="47" t="s">
         <v>54</v>
       </c>
-      <c r="D50" s="53" t="s">
+      <c r="D50" s="48" t="s">
         <v>55</v>
       </c>
-      <c r="E50" s="40">
+      <c r="E50" s="36">
         <v>95.554434968172885</v>
       </c>
-      <c r="F50" s="40">
+      <c r="F50" s="36">
         <v>81.865643703186961</v>
       </c>
-      <c r="G50" s="41">
+      <c r="G50" s="37">
         <v>87.977413403662496</v>
       </c>
-      <c r="H50" s="31"/>
-    </row>
-    <row r="51" spans="3:8" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="C51" s="60" t="s">
+      <c r="H50" s="29"/>
+    </row>
+    <row r="51" spans="3:8" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="C51" s="55" t="s">
         <v>56</v>
       </c>
-      <c r="D51" s="53" t="s">
+      <c r="D51" s="48" t="s">
         <v>57</v>
       </c>
-      <c r="E51" s="62">
+      <c r="E51" s="57">
         <v>333</v>
       </c>
-      <c r="F51" s="62">
+      <c r="F51" s="57">
         <v>323</v>
       </c>
-      <c r="G51" s="63">
+      <c r="G51" s="58">
         <v>656</v>
       </c>
-      <c r="H51" s="31"/>
-    </row>
-    <row r="52" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C52" s="72" t="s">
+      <c r="H51" s="29"/>
+    </row>
+    <row r="52" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C52" s="67" t="s">
         <v>32</v>
       </c>
-      <c r="D52" s="73"/>
-      <c r="E52" s="64"/>
-      <c r="F52" s="64"/>
-      <c r="G52" s="64"/>
-      <c r="H52" s="44"/>
-    </row>
-    <row r="53" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C53" s="74" t="s">
+      <c r="D52" s="68"/>
+      <c r="E52" s="59"/>
+      <c r="F52" s="59"/>
+      <c r="G52" s="59"/>
+      <c r="H52" s="40"/>
+    </row>
+    <row r="53" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C53" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="D53" s="75" t="s">
+      <c r="D53" s="70" t="s">
         <v>51</v>
       </c>
-      <c r="E53" s="65">
+      <c r="E53" s="60">
         <v>700.2276580423146</v>
       </c>
-      <c r="F53" s="65">
+      <c r="F53" s="60">
         <v>800.17804231053913</v>
       </c>
-      <c r="G53" s="66">
+      <c r="G53" s="61">
         <v>750.84301982153386</v>
       </c>
       <c r="H53" s="19"/>
     </row>
-    <row r="54" spans="3:8" ht="42.75" x14ac:dyDescent="0.2">
-      <c r="C54" s="76" t="s">
+    <row r="54" spans="3:8" ht="41.4" x14ac:dyDescent="0.25">
+      <c r="C54" s="71" t="s">
         <v>33</v>
       </c>
-      <c r="D54" s="77" t="s">
+      <c r="D54" s="72" t="s">
         <v>34</v>
       </c>
-      <c r="E54" s="67">
+      <c r="E54" s="62">
         <v>2.7436813556600068</v>
       </c>
-      <c r="F54" s="67">
+      <c r="F54" s="62">
         <v>2.7433759999576579</v>
       </c>
-      <c r="G54" s="68">
+      <c r="G54" s="63">
         <v>2.74351607550238</v>
       </c>
-      <c r="H54" s="31"/>
-    </row>
-    <row r="55" spans="3:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="C55" s="74" t="s">
+      <c r="H54" s="29"/>
+    </row>
+    <row r="55" spans="3:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="C55" s="69" t="s">
         <v>35</v>
       </c>
-      <c r="D55" s="75" t="s">
+      <c r="D55" s="70" t="s">
         <v>36</v>
       </c>
-      <c r="E55" s="59">
+      <c r="E55" s="54">
         <v>2.58</v>
       </c>
-      <c r="F55" s="49"/>
-      <c r="G55" s="56">
+      <c r="F55" s="45"/>
+      <c r="G55" s="51">
         <v>2.58</v>
       </c>
       <c r="H55" s="18"/>
     </row>
-    <row r="56" spans="3:8" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C56" s="54" t="s">
+    <row r="56" spans="3:8" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C56" s="49" t="s">
         <v>52</v>
       </c>
-      <c r="D56" s="55" t="s">
+      <c r="D56" s="50" t="s">
         <v>53</v>
       </c>
-      <c r="E56" s="69">
+      <c r="E56" s="64">
         <v>9.873282781508065</v>
       </c>
-      <c r="F56" s="48"/>
-      <c r="G56" s="70">
+      <c r="F56" s="44"/>
+      <c r="G56" s="65">
         <v>9.873282781508065</v>
       </c>
       <c r="H56" s="6"/>
     </row>
-    <row r="58" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="E58" s="61"/>
-      <c r="F58" s="61"/>
+    <row r="58" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="E58" s="56"/>
+      <c r="F58" s="56"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>